<commit_message>
Inclusao de novos produtos (Pacocas e Farinha) e ordenacao alfabetica de itens
- Cadastro de Pacoca Rolha Tigre nas apresentacoes 60x100g, 24x300g e 12x504g com fotos e precos

- Cadastro de Farinha de Mandioca Grossa Tigre 25x400g e inclusao de foto

- Classificacao automatica de Pacocas na categoria Doces no app

- Ordenacao alfabetica dos produtos dentro de cada categoria na interface do usuario
</commit_message>
<xml_diff>
--- a/Produtos_tigre_pedido_exemplo.xlsx
+++ b/Produtos_tigre_pedido_exemplo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1373,11 +1373,11 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>FARINHA DE MANDIOCA FINA TIGRE 10X1KG</t>
+          <t>FARINHA DE MANDIOCA GROSSA TIGRE 25X400GR</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>6.89</v>
+        <v>2.76</v>
       </c>
       <c r="C40" t="n">
         <v>68.90000000000001</v>
@@ -1385,46 +1385,52 @@
       <c r="D40" t="n">
         <v>10</v>
       </c>
-      <c r="E40" t="n">
-        <v>10</v>
-      </c>
       <c r="F40" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>689</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>FARINHA DE ROSCA TIGRE 24X400GR</t>
+          <t>FARINHA DE MANDIOCA FINA TIGRE 10X1KG</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>4.43</v>
+        <v>6.89</v>
       </c>
       <c r="C41" t="n">
-        <v>106.32</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="D41" t="n">
-        <v>9.6</v>
+        <v>10</v>
+      </c>
+      <c r="E41" t="n">
+        <v>10</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>689</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>FAROFA TEMPERADA TIGRE 20X500GR(EM FALTA)</t>
-        </is>
+          <t>FARINHA DE ROSCA TIGRE 24X400GR</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="C42" t="n">
+        <v>106.32</v>
       </c>
       <c r="D42" t="n">
-        <v>10</v>
+        <v>9.6</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
@@ -1436,14 +1442,8 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FÚBA DE MILHO 25X400GR</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>2.43</v>
-      </c>
-      <c r="C43" t="n">
-        <v>60.75</v>
+          <t>FAROFA TEMPERADA TIGRE 20X500GR(EM FALTA)</t>
+        </is>
       </c>
       <c r="D43" t="n">
         <v>10</v>
@@ -1458,101 +1458,101 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GRAO DE BICO TIGRE 25X400GRS</t>
+          <t>FÚBA DE MILHO 25X400GR</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>4.32</v>
+        <v>2.43</v>
       </c>
       <c r="C44" t="n">
-        <v>108</v>
+        <v>60.75</v>
       </c>
       <c r="D44" t="n">
         <v>10</v>
       </c>
-      <c r="E44" t="n">
-        <v>1</v>
-      </c>
       <c r="F44" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GIRASSOL MIUDO TIGRE 20X500GR</t>
+          <t>GRAO DE BICO TIGRE 25X400GRS</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>4.19</v>
+        <v>4.32</v>
       </c>
       <c r="C45" t="n">
-        <v>83.8</v>
+        <v>108</v>
       </c>
       <c r="D45" t="n">
         <v>10</v>
       </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LENTILHA TIGRE 25X400GR</t>
+          <t>GIRASSOL MIUDO TIGRE 20X500GR</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>4.32</v>
+        <v>4.19</v>
       </c>
       <c r="C46" t="n">
-        <v>108</v>
+        <v>83.8</v>
       </c>
       <c r="D46" t="n">
         <v>10</v>
       </c>
-      <c r="E46" t="n">
-        <v>2</v>
-      </c>
       <c r="F46" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>216</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>POLVILHO AZEDO TIGRE 20X500GR</t>
+          <t>LENTILHA TIGRE 25X400GR</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>4.46</v>
+        <v>4.32</v>
       </c>
       <c r="C47" t="n">
-        <v>89.2</v>
+        <v>108</v>
       </c>
       <c r="D47" t="n">
         <v>10</v>
       </c>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
       <c r="F47" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G47" t="n">
-        <v>0</v>
+        <v>216</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>POLVILHO DOCE TIGRE 20X500GR</t>
+          <t>POLVILHO AZEDO TIGRE 20X500GR</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1574,182 +1574,270 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MILHO P/ PIPOCA TIGRE 25X400GR</t>
+          <t>POLVILHO DOCE TIGRE 20X500GR</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2.77</v>
+        <v>4.46</v>
       </c>
       <c r="C49" t="n">
-        <v>69.25</v>
+        <v>89.2</v>
       </c>
       <c r="D49" t="n">
         <v>10</v>
       </c>
-      <c r="E49" t="n">
-        <v>144</v>
-      </c>
       <c r="F49" t="n">
-        <v>1440</v>
+        <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>9972</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>RAPADURA MINEIRA JR 5X600GR</t>
+          <t>MILHO P/ PIPOCA TIGRE 25X400GR</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>6.97</v>
+        <v>2.77</v>
       </c>
       <c r="C50" t="n">
-        <v>34.85</v>
+        <v>69.25</v>
       </c>
       <c r="D50" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>12</v>
+        <v>144</v>
       </c>
       <c r="F50" t="n">
-        <v>36</v>
+        <v>1440</v>
       </c>
       <c r="G50" t="n">
-        <v>418.2</v>
+        <v>9972</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SAL DO HIMALAIA 10X1KG</t>
+          <t>RAPADURA MINEIRA JR 5X600GR</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>6.28</v>
+        <v>6.97</v>
       </c>
       <c r="C51" t="n">
-        <v>62.8</v>
+        <v>34.85</v>
       </c>
       <c r="D51" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E51" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F51" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="G51" t="n">
-        <v>628</v>
+        <v>418.2</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SOJA TIGRE 25X400GRS</t>
+          <t>SAL DO HIMALAIA 10X1KG</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2.82</v>
+        <v>6.28</v>
       </c>
       <c r="C52" t="n">
-        <v>70.5</v>
+        <v>62.8</v>
       </c>
       <c r="D52" t="n">
         <v>10</v>
       </c>
+      <c r="E52" t="n">
+        <v>10</v>
+      </c>
       <c r="F52" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G52" t="n">
-        <v>0</v>
+        <v>628</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SAGU TIGRE 20X500GR</t>
+          <t>SOJA TIGRE 25X400GRS</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>4.87</v>
+        <v>2.82</v>
       </c>
       <c r="C53" t="n">
-        <v>97.40000000000001</v>
+        <v>70.5</v>
       </c>
       <c r="D53" t="n">
         <v>10</v>
       </c>
-      <c r="E53" t="n">
-        <v>2</v>
-      </c>
       <c r="F53" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>194.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TRIGO P/ KIBE TIGRE 20X500GR</t>
+          <t>SAGU TIGRE 20X500GR</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>3.3</v>
+        <v>4.87</v>
       </c>
       <c r="C54" t="n">
-        <v>66</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="D54" t="n">
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="F54" t="n">
-        <v>110</v>
+        <v>20</v>
       </c>
       <c r="G54" t="n">
-        <v>726</v>
+        <v>194.8</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TAPIOCA GRANULADA 20X500GR</t>
+          <t>TRIGO P/ KIBE TIGRE 20X500GR</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>5</v>
+        <v>3.3</v>
       </c>
       <c r="C55" t="n">
-        <v>100</v>
+        <v>66</v>
       </c>
       <c r="D55" t="n">
         <v>10</v>
       </c>
+      <c r="E55" t="n">
+        <v>11</v>
+      </c>
       <c r="F55" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="G55" t="n">
-        <v>0</v>
+        <v>726</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>TAPIOCA GRANULADA 20X500GR</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>5</v>
+      </c>
+      <c r="C56" t="n">
+        <v>100</v>
+      </c>
+      <c r="D56" t="n">
+        <v>10</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>PAÇOCA ROLHA TIGRE 60X100GR</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="C57" t="n">
+        <v>110.71</v>
+      </c>
+      <c r="D57" t="n">
+        <v>6</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>PAÇOCA ROLHA TIGRE 24X300GR</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="C58" t="n">
+        <v>159.18</v>
+      </c>
+      <c r="D58" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>PAÇOCA ROLHA TIGRE 12X504GR</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="C59" t="n">
+        <v>99.44</v>
+      </c>
+      <c r="D59" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>TOTAL GRÃOS</t>
         </is>
       </c>
-      <c r="F56" t="n">
+      <c r="F60" t="n">
         <v>14928</v>
       </c>
-      <c r="G56" t="n">
+      <c r="G60" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>